<commit_message>
Add servicing and lubrication tasks
</commit_message>
<xml_diff>
--- a/Control_de_aeronavegabilidad2026.xlsx
+++ b/Control_de_aeronavegabilidad2026.xlsx
@@ -1744,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="26.86" customWidth="1" style="48" min="1" max="1"/>
@@ -2580,38 +2580,27 @@
       <c r="L32" s="52" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="48">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="0" t="inlineStr">
         <is>
           <t>Air data systems tightness test</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="0" t="n">
         <v>300</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" s="0" t="n">
         <v>1095</v>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="K33" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.222</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="48">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="0" t="inlineStr">
         <is>
           <t>ELT visual inspection and operational test</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>100</v>
-      </c>
-      <c r="D34" t="n">
-        <v>180</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.211</t>
         </is>
       </c>
     </row>
@@ -2631,7 +2620,7 @@
       <c r="H36" s="51" t="n"/>
       <c r="I36" s="51" t="n"/>
       <c r="J36" s="51" t="n"/>
-      <c r="K36" s="51" t="n"/>
+      <c r="K36" s="52" t="n"/>
       <c r="L36" s="52" t="n"/>
     </row>
     <row r="37" ht="31.5" customHeight="1" s="48">
@@ -2725,17 +2714,15 @@
     <row r="39" ht="15.75" customHeight="1" s="48">
       <c r="A39" s="25" t="inlineStr">
         <is>
-          <t>Lubricate Área 100</t>
-        </is>
-      </c>
-      <c r="B39" s="28" t="inlineStr">
-        <is>
-          <t>50, 100, 2000</t>
-        </is>
+          <t>Drain oil system / filter / crankcase strainer</t>
+        </is>
+      </c>
+      <c r="B39" s="28" t="n">
+        <v>50</v>
       </c>
       <c r="C39" s="26" t="n"/>
       <c r="D39" s="26" t="n">
-        <v>365</v>
+        <v>120</v>
       </c>
       <c r="E39" s="25" t="n"/>
       <c r="F39" s="25" t="n"/>
@@ -2743,33 +2730,47 @@
       <c r="H39" s="25" t="n"/>
       <c r="I39" s="25" t="n"/>
       <c r="J39" s="25" t="n"/>
-      <c r="K39" s="26" t="n"/>
+      <c r="K39" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203 ATA 12-10</t>
+        </is>
+      </c>
       <c r="L39" s="52" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="48">
-      <c r="A40" s="25" t="n"/>
-      <c r="B40" s="28" t="n"/>
+      <c r="A40" s="25" t="inlineStr">
+        <is>
+          <t>Drain fuel tanks and fuel system / ventilate</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="n">
+        <v>2000</v>
+      </c>
       <c r="C40" s="26" t="n"/>
-      <c r="D40" s="26" t="n"/>
+      <c r="D40" s="26" t="n">
+        <v>365</v>
+      </c>
       <c r="E40" s="25" t="n"/>
       <c r="F40" s="25" t="n"/>
       <c r="G40" s="25" t="n"/>
       <c r="H40" s="25" t="n"/>
       <c r="I40" s="25" t="n"/>
       <c r="J40" s="25" t="n"/>
-      <c r="K40" s="26" t="n"/>
+      <c r="K40" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203 ATA 12-10</t>
+        </is>
+      </c>
       <c r="L40" s="26" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="48">
       <c r="A41" s="29" t="inlineStr">
         <is>
-          <t>Clean exterior surface &amp; de Engine (12-20)</t>
-        </is>
-      </c>
-      <c r="B41" s="28" t="inlineStr">
-        <is>
-          <t>100, 2000</t>
-        </is>
+          <t>Clean exterior surface / inspect corrosion</t>
+        </is>
+      </c>
+      <c r="B41" s="28" t="n">
+        <v>100</v>
       </c>
       <c r="C41" s="26" t="n"/>
       <c r="D41" s="26" t="n">
@@ -2781,15 +2782,115 @@
       <c r="H41" s="25" t="n"/>
       <c r="I41" s="25" t="n"/>
       <c r="J41" s="25" t="n"/>
-      <c r="K41" s="26" t="n"/>
+      <c r="K41" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203 ATA 12-20</t>
+        </is>
+      </c>
       <c r="L41" s="52" t="n"/>
     </row>
-    <row r="42" ht="15.75" customHeight="1" s="48"/>
-    <row r="43" ht="15.75" customHeight="1" s="48"/>
-    <row r="44" ht="15.75" customHeight="1" s="48"/>
-    <row r="45" ht="15.75" customHeight="1" s="48"/>
-    <row r="46" ht="15.75" customHeight="1" s="48"/>
-    <row r="47" ht="15.75" customHeight="1" s="48"/>
+    <row r="42" ht="15.75" customHeight="1" s="48">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Clean engine</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D42" t="n">
+        <v>365</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203 ATA 12-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="48">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Anticorrosion/lubrication cockpit-fuselage &amp; landing gear</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>50</v>
+      </c>
+      <c r="D43" t="n">
+        <v>365</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203-204 ATA 20-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="48">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Anticorrosion/lubrication stabilizers/wings/engine compartment</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>100</v>
+      </c>
+      <c r="D44" t="n">
+        <v>365</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.204 ATA 20-00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="48">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Lubricate bearings and wheel axles</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D45" t="n">
+        <v>365</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.219 ATA 32-40</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="48">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Lubricate door locking mechanisms</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.224 ATA 52-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="48">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Lubricate inside elevator balancing boom</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2000</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.227 ATA 55-20</t>
+        </is>
+      </c>
+    </row>
     <row r="48" ht="15.75" customHeight="1" s="48"/>
     <row r="49" ht="15.75" customHeight="1" s="48"/>
     <row r="50" ht="15.75" customHeight="1" s="48"/>

</xml_diff>

<commit_message>
Add life limit and TBO components
</commit_message>
<xml_diff>
--- a/Control_de_aeronavegabilidad2026.xlsx
+++ b/Control_de_aeronavegabilidad2026.xlsx
@@ -2790,102 +2790,102 @@
       <c r="L41" s="52" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="48">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="0" t="inlineStr">
         <is>
           <t>Clean engine</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="D42" t="n">
+      <c r="D42" s="0" t="n">
         <v>365</v>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203 ATA 12-20</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="48">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="0" t="inlineStr">
         <is>
           <t>Anticorrosion/lubrication cockpit-fuselage &amp; landing gear</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="0" t="n">
         <v>50</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D43" s="0" t="n">
         <v>365</v>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.203-204 ATA 20-00</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="48">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="0" t="inlineStr">
         <is>
           <t>Anticorrosion/lubrication stabilizers/wings/engine compartment</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="0" t="n">
         <v>100</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D44" s="0" t="n">
         <v>365</v>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.204 ATA 20-00</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="48">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="0" t="inlineStr">
         <is>
           <t>Lubricate bearings and wheel axles</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D45" s="0" t="n">
         <v>365</v>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.219 ATA 32-40</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="48">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="0" t="inlineStr">
         <is>
           <t>Lubricate door locking mechanisms</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.224 ATA 52-10</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="48">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="0" t="inlineStr">
         <is>
           <t>Lubricate inside elevator balancing boom</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="0" t="n">
         <v>2000</v>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB 10 MM Rev.18, 05-20-01 p.227 ATA 55-20</t>
         </is>
@@ -3902,7 +3902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22.86" customWidth="1" style="48" min="1" max="2"/>
@@ -4110,18 +4110,20 @@
     <row r="8">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>MOTOR</t>
+          <t>Motor</t>
         </is>
       </c>
       <c r="B8" s="25" t="inlineStr">
         <is>
-          <t>Lycoming IO-360-RRR</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="n"/>
+          <t>Lycoming O-360-A1AD</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D8" s="26" t="n"/>
       <c r="E8" s="26" t="n">
-        <v>180</v>
+        <v>4380</v>
       </c>
       <c r="F8" s="25" t="n"/>
       <c r="G8" s="25" t="n"/>
@@ -4129,37 +4131,65 @@
       <c r="I8" s="25" t="n"/>
       <c r="J8" s="25" t="n"/>
       <c r="K8" s="25" t="n"/>
-      <c r="L8" s="25" t="n"/>
-      <c r="M8" s="26" t="n"/>
+      <c r="L8" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M8" s="26" t="inlineStr">
+        <is>
+          <t>Lycoming SI 1009BE p.2,p.3; SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N8" s="52" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>FILTRO DEL AIRE</t>
-        </is>
-      </c>
-      <c r="B9" s="25" t="n"/>
-      <c r="C9" s="26" t="n"/>
+          <t>Alternator</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>ALX 8421 / ALX 8521 / ALU 8421</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D9" s="26" t="n"/>
-      <c r="E9" s="26" t="n"/>
+      <c r="E9" s="26" t="n">
+        <v>4380</v>
+      </c>
       <c r="F9" s="25" t="n"/>
       <c r="G9" s="25" t="n"/>
       <c r="H9" s="25" t="n"/>
       <c r="I9" s="25" t="n"/>
       <c r="J9" s="25" t="n"/>
       <c r="K9" s="25" t="n"/>
-      <c r="L9" s="25" t="n"/>
-      <c r="M9" s="26" t="n"/>
+      <c r="L9" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M9" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.1</t>
+        </is>
+      </c>
       <c r="N9" s="52" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETO </t>
-        </is>
-      </c>
-      <c r="B10" s="25" t="n"/>
+          <t>Propeller</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Hartzell HC-C2YK-1BF/F7666 A-2</t>
+        </is>
+      </c>
       <c r="C10" s="26" t="n"/>
       <c r="D10" s="26" t="n"/>
       <c r="E10" s="26" t="n"/>
@@ -4169,150 +4199,260 @@
       <c r="I10" s="25" t="n"/>
       <c r="J10" s="25" t="n"/>
       <c r="K10" s="25" t="n"/>
-      <c r="L10" s="25" t="n"/>
-      <c r="M10" s="26" t="n"/>
+      <c r="L10" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M10" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N10" s="52" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>BOMBA DE COMBUSTIBLE</t>
-        </is>
-      </c>
-      <c r="B11" s="25" t="n"/>
-      <c r="C11" s="26" t="n"/>
+          <t>Propeller governor</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Hartzell F4-26</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D11" s="26" t="n"/>
-      <c r="E11" s="26" t="n"/>
+      <c r="E11" s="26" t="n">
+        <v>4380</v>
+      </c>
       <c r="F11" s="25" t="n"/>
       <c r="G11" s="25" t="n"/>
       <c r="H11" s="25" t="n"/>
       <c r="I11" s="25" t="n"/>
       <c r="J11" s="25" t="n"/>
       <c r="K11" s="25" t="n"/>
-      <c r="L11" s="25" t="n"/>
-      <c r="M11" s="26" t="n"/>
+      <c r="L11" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M11" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N11" s="52" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>PUESTA EN MARCHA</t>
-        </is>
-      </c>
-      <c r="B12" s="25" t="n"/>
-      <c r="C12" s="26" t="n"/>
+          <t>Carburetor</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>Marvel 71098 MA-4-5</t>
+        </is>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D12" s="26" t="n"/>
-      <c r="E12" s="26" t="n"/>
+      <c r="E12" s="26" t="n">
+        <v>4380</v>
+      </c>
       <c r="F12" s="25" t="n"/>
       <c r="G12" s="25" t="n"/>
       <c r="H12" s="25" t="n"/>
       <c r="I12" s="25" t="n"/>
       <c r="J12" s="25" t="n"/>
       <c r="K12" s="25" t="n"/>
-      <c r="L12" s="25" t="n"/>
-      <c r="M12" s="26" t="n"/>
+      <c r="L12" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M12" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N12" s="52" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>BOMBA  DE VACIO</t>
-        </is>
-      </c>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="26" t="n"/>
+          <t>Dual magneto</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>TCM D4LN3000</t>
+        </is>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D13" s="26" t="n"/>
-      <c r="E13" s="26" t="n"/>
+      <c r="E13" s="26" t="n">
+        <v>1460</v>
+      </c>
       <c r="F13" s="25" t="n"/>
       <c r="G13" s="25" t="n"/>
       <c r="H13" s="25" t="n"/>
       <c r="I13" s="25" t="n"/>
       <c r="J13" s="25" t="n"/>
       <c r="K13" s="25" t="n"/>
-      <c r="L13" s="25" t="n"/>
-      <c r="M13" s="26" t="n"/>
+      <c r="L13" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M13" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N13" s="52" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>CINTURONES</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="26" t="n"/>
+          <t>Starter</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>MZ 4222 / Lycoming LW15571</t>
+        </is>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>2000</v>
+      </c>
       <c r="D14" s="26" t="n"/>
-      <c r="E14" s="26" t="n"/>
+      <c r="E14" s="26" t="n">
+        <v>4380</v>
+      </c>
       <c r="F14" s="25" t="n"/>
       <c r="G14" s="25" t="n"/>
       <c r="H14" s="25" t="n"/>
       <c r="I14" s="25" t="n"/>
       <c r="J14" s="25" t="n"/>
       <c r="K14" s="25" t="n"/>
-      <c r="L14" s="25" t="n"/>
-      <c r="M14" s="26" t="n"/>
+      <c r="L14" s="25" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="M14" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.4</t>
+        </is>
+      </c>
       <c r="N14" s="52" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>ALTERNADOR</t>
-        </is>
-      </c>
-      <c r="B15" s="25" t="n"/>
+          <t>ELT battery assembly</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>As installed</t>
+        </is>
+      </c>
       <c r="C15" s="26" t="n"/>
       <c r="D15" s="26" t="n"/>
-      <c r="E15" s="26" t="n"/>
+      <c r="E15" s="26" t="n">
+        <v>1460</v>
+      </c>
       <c r="F15" s="25" t="n"/>
       <c r="G15" s="25" t="n"/>
       <c r="H15" s="25" t="n"/>
       <c r="I15" s="25" t="n"/>
       <c r="J15" s="25" t="n"/>
       <c r="K15" s="25" t="n"/>
-      <c r="L15" s="25" t="n"/>
-      <c r="M15" s="26" t="n"/>
+      <c r="L15" s="25" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M15" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.1-2</t>
+        </is>
+      </c>
       <c r="N15" s="52" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>CARBURADOR</t>
-        </is>
-      </c>
-      <c r="B16" s="25" t="n"/>
+          <t>ELT seals</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>ELT90/91/96/97 seals</t>
+        </is>
+      </c>
       <c r="C16" s="25" t="n"/>
       <c r="D16" s="25" t="n"/>
-      <c r="E16" s="25" t="n"/>
+      <c r="E16" s="25" t="n">
+        <v>4380</v>
+      </c>
       <c r="F16" s="25" t="n"/>
       <c r="G16" s="25" t="n"/>
       <c r="H16" s="25" t="n"/>
       <c r="I16" s="25" t="n"/>
       <c r="J16" s="25" t="n"/>
       <c r="K16" s="25" t="n"/>
-      <c r="L16" s="25" t="n"/>
-      <c r="M16" s="26" t="n"/>
+      <c r="L16" s="25" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M16" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.2</t>
+        </is>
+      </c>
       <c r="N16" s="52" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="48">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>HÉLICE</t>
-        </is>
-      </c>
-      <c r="B17" s="25" t="n"/>
+          <t>Fire extinguisher</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>MAIP/AREOFEU/LHOTELLIER as installed</t>
+        </is>
+      </c>
       <c r="C17" s="25" t="n"/>
       <c r="D17" s="25" t="n"/>
-      <c r="E17" s="25" t="n"/>
+      <c r="E17" s="25" t="n">
+        <v>3650</v>
+      </c>
       <c r="F17" s="25" t="n"/>
       <c r="G17" s="25" t="n"/>
       <c r="H17" s="25" t="n"/>
       <c r="I17" s="25" t="n"/>
       <c r="J17" s="25" t="n"/>
       <c r="K17" s="25" t="n"/>
-      <c r="L17" s="25" t="n"/>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t>Discard/Inspection</t>
+        </is>
+      </c>
       <c r="M17" s="55" t="inlineStr">
         <is>
-          <t>HARTZELL Service Letter HC-SL-61-61Y</t>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.3 TR006.05</t>
         </is>
       </c>
       <c r="N17" s="52" t="n"/>
@@ -4320,268 +4460,315 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>GOVERNOR</t>
-        </is>
-      </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
+          <t>Vacuum system filter</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>AIRBORNE 1J4-7</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>500</v>
+      </c>
       <c r="D18" s="25" t="n"/>
-      <c r="E18" s="25" t="n"/>
+      <c r="E18" s="25" t="n">
+        <v>365</v>
+      </c>
       <c r="F18" s="25" t="n"/>
       <c r="G18" s="25" t="n"/>
       <c r="H18" s="25" t="n"/>
       <c r="I18" s="25" t="n"/>
       <c r="J18" s="25" t="n"/>
       <c r="K18" s="25" t="n"/>
-      <c r="L18" s="25" t="n"/>
-      <c r="M18" s="26" t="n"/>
+      <c r="L18" s="25" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M18" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.3</t>
+        </is>
+      </c>
       <c r="N18" s="52" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>Cinturones</t>
-        </is>
-      </c>
-      <c r="B19" s="25" t="n"/>
+          <t>Emergency vacuum pump</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>AIRBORNE 4A3-1 14V</t>
+        </is>
+      </c>
       <c r="C19" s="25" t="n"/>
       <c r="D19" s="25" t="n"/>
-      <c r="E19" s="25" t="n"/>
+      <c r="E19" s="25" t="n">
+        <v>3650</v>
+      </c>
       <c r="F19" s="25" t="n"/>
       <c r="G19" s="25" t="n"/>
       <c r="H19" s="25" t="n"/>
       <c r="I19" s="25" t="n"/>
       <c r="J19" s="25" t="n"/>
       <c r="K19" s="25" t="n"/>
-      <c r="L19" s="25" t="n"/>
-      <c r="M19" s="26" t="n"/>
+      <c r="L19" s="25" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M19" s="26" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.3</t>
+        </is>
+      </c>
       <c r="N19" s="52" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="n"/>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="25" t="n"/>
-      <c r="D20" s="25" t="n"/>
-      <c r="E20" s="25" t="n"/>
-      <c r="F20" s="25" t="n"/>
-      <c r="G20" s="25" t="n"/>
-      <c r="H20" s="25" t="n"/>
-      <c r="I20" s="25" t="n"/>
-      <c r="J20" s="25" t="n"/>
-      <c r="K20" s="25" t="n"/>
-      <c r="L20" s="25" t="n"/>
-      <c r="M20" s="26" t="n"/>
-      <c r="N20" s="52" t="n"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="48"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Access door latches</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TB10 25012102</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1" s="48">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Teflon hoses</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Teflon hoses</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>On Condition</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.5-9</t>
+        </is>
+      </c>
+    </row>
     <row r="22" ht="15.75" customHeight="1" s="48">
-      <c r="A22" s="54" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Fuel selector filter/drain hose</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TB10 52035114</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E22" t="n">
+        <v>3650</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="48">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Elastomer/rubber/vinyl hoses</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Assorted</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>3650</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Discard</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>SOCATA TB10 MM Rev.18 05-10-00 p.5-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="48"/>
+    <row r="25" ht="15.75" customHeight="1" s="48">
+      <c r="A25" s="25" t="n"/>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="25" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+      <c r="K25" s="25" t="n"/>
+      <c r="L25" s="25" t="n"/>
+      <c r="M25" s="26" t="n"/>
+      <c r="N25" s="52" t="n"/>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="48"/>
+    <row r="27" ht="15.75" customHeight="1" s="48">
+      <c r="A27" s="54" t="inlineStr">
         <is>
           <t>AIRWORTHINESS LIMITATIONS Items</t>
         </is>
       </c>
-      <c r="B22" s="51" t="n"/>
-      <c r="C22" s="51" t="n"/>
-      <c r="D22" s="51" t="n"/>
-      <c r="E22" s="51" t="n"/>
-      <c r="F22" s="51" t="n"/>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="51" t="n"/>
-      <c r="I22" s="51" t="n"/>
-      <c r="J22" s="51" t="n"/>
-      <c r="K22" s="51" t="n"/>
-      <c r="L22" s="51" t="n"/>
-      <c r="M22" s="51" t="n"/>
-      <c r="N22" s="52" t="n"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="48">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="18" t="inlineStr">
+      <c r="B27" s="51" t="n"/>
+      <c r="C27" s="51" t="n"/>
+      <c r="D27" s="51" t="n"/>
+      <c r="E27" s="51" t="n"/>
+      <c r="F27" s="51" t="n"/>
+      <c r="G27" s="51" t="n"/>
+      <c r="H27" s="51" t="n"/>
+      <c r="I27" s="51" t="n"/>
+      <c r="J27" s="51" t="n"/>
+      <c r="K27" s="51" t="n"/>
+      <c r="L27" s="51" t="n"/>
+      <c r="M27" s="51" t="n"/>
+      <c r="N27" s="52" t="n"/>
+    </row>
+    <row r="28" ht="15.75" customHeight="1" s="48">
+      <c r="A28" s="13" t="n"/>
+      <c r="B28" s="13" t="n"/>
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>Interval /TBO</t>
         </is>
       </c>
-      <c r="D23" s="51" t="n"/>
-      <c r="E23" s="52" t="n"/>
-      <c r="F23" s="47" t="inlineStr">
+      <c r="D28" s="51" t="n"/>
+      <c r="E28" s="52" t="n"/>
+      <c r="F28" s="47" t="inlineStr">
         <is>
           <t>Interval FH/ CyC/Ldgs</t>
         </is>
       </c>
-      <c r="G23" s="51" t="n"/>
-      <c r="H23" s="52" t="n"/>
-      <c r="I23" s="47" t="inlineStr">
+      <c r="G28" s="51" t="n"/>
+      <c r="H28" s="52" t="n"/>
+      <c r="I28" s="47" t="inlineStr">
         <is>
           <t>Calendar</t>
         </is>
       </c>
-      <c r="J23" s="51" t="n"/>
-      <c r="K23" s="52" t="n"/>
-      <c r="L23" s="31" t="n"/>
-      <c r="M23" s="47" t="inlineStr">
+      <c r="J28" s="51" t="n"/>
+      <c r="K28" s="52" t="n"/>
+      <c r="L28" s="31" t="n"/>
+      <c r="M28" s="47" t="inlineStr">
         <is>
           <t>Applicable ICA reference</t>
         </is>
       </c>
-      <c r="N23" s="52" t="n"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="48">
-      <c r="A24" s="18" t="inlineStr">
+      <c r="N28" s="52" t="n"/>
+    </row>
+    <row r="29" ht="15.75" customHeight="1" s="48">
+      <c r="A29" s="18" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C29" s="19" t="inlineStr">
         <is>
           <t>FH</t>
         </is>
       </c>
-      <c r="D24" s="20" t="inlineStr">
+      <c r="D29" s="20" t="inlineStr">
         <is>
           <t>Ldg/Cycle</t>
         </is>
       </c>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F29" s="21" t="inlineStr">
         <is>
           <t>Performed</t>
         </is>
       </c>
-      <c r="G24" s="22" t="inlineStr">
+      <c r="G29" s="22" t="inlineStr">
         <is>
           <t>Next due</t>
         </is>
       </c>
-      <c r="H24" s="23" t="inlineStr">
+      <c r="H29" s="23" t="inlineStr">
         <is>
           <t>to go</t>
         </is>
       </c>
-      <c r="I24" s="21" t="inlineStr">
+      <c r="I29" s="21" t="inlineStr">
         <is>
           <t>Performed</t>
         </is>
       </c>
-      <c r="J24" s="22" t="inlineStr">
+      <c r="J29" s="22" t="inlineStr">
         <is>
           <t>Next due</t>
         </is>
       </c>
-      <c r="K24" s="23" t="inlineStr">
+      <c r="K29" s="23" t="inlineStr">
         <is>
           <t>to go</t>
         </is>
       </c>
-      <c r="L24" s="32" t="inlineStr">
+      <c r="L29" s="32" t="inlineStr">
         <is>
           <t>Tipe of Task (OH, Discard, On Condition)</t>
         </is>
       </c>
-      <c r="M24" s="26" t="inlineStr">
+      <c r="M29" s="26" t="inlineStr">
         <is>
           <t>Document / Revision</t>
         </is>
       </c>
-      <c r="N24" s="52" t="n"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="48">
-      <c r="A25" s="56" t="inlineStr">
-        <is>
-          <t>STRUCTURE SERVICE LIFE</t>
-        </is>
-      </c>
-      <c r="B25" s="51" t="n"/>
-      <c r="C25" s="51" t="n"/>
-      <c r="D25" s="51" t="n"/>
-      <c r="E25" s="51" t="n"/>
-      <c r="F25" s="51" t="n"/>
-      <c r="G25" s="51" t="n"/>
-      <c r="H25" s="51" t="n"/>
-      <c r="I25" s="51" t="n"/>
-      <c r="J25" s="51" t="n"/>
-      <c r="K25" s="51" t="n"/>
-      <c r="L25" s="51" t="n"/>
-      <c r="M25" s="51" t="n"/>
-      <c r="N25" s="52" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="48">
-      <c r="A26" s="25" t="n"/>
-      <c r="B26" s="25" t="n"/>
-      <c r="C26" s="26" t="n"/>
-      <c r="D26" s="26" t="n"/>
-      <c r="E26" s="26" t="n"/>
-      <c r="F26" s="25" t="n"/>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="25" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="n"/>
-      <c r="M26" s="26" t="n"/>
-      <c r="N26" s="52" t="n"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="48">
-      <c r="A27" s="25" t="n"/>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="26" t="n"/>
-      <c r="D27" s="26" t="n"/>
-      <c r="E27" s="26" t="n"/>
-      <c r="F27" s="25" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="25" t="n"/>
-      <c r="K27" s="25" t="n"/>
-      <c r="L27" s="25" t="n"/>
-      <c r="M27" s="26" t="n"/>
-      <c r="N27" s="52" t="n"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="48">
-      <c r="A28" s="25" t="n"/>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="26" t="n"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
-      <c r="F28" s="25" t="n"/>
-      <c r="G28" s="25" t="n"/>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
-      <c r="J28" s="25" t="n"/>
-      <c r="K28" s="25" t="n"/>
-      <c r="L28" s="25" t="n"/>
-      <c r="M28" s="26" t="n"/>
-      <c r="N28" s="52" t="n"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" s="48">
-      <c r="A29" s="25" t="n"/>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="26" t="n"/>
-      <c r="D29" s="26" t="n"/>
-      <c r="E29" s="26" t="n"/>
-      <c r="F29" s="25" t="n"/>
-      <c r="G29" s="25" t="n"/>
-      <c r="H29" s="25" t="n"/>
-      <c r="I29" s="25" t="n"/>
-      <c r="J29" s="25" t="n"/>
-      <c r="K29" s="25" t="n"/>
-      <c r="L29" s="25" t="n"/>
-      <c r="M29" s="26" t="n"/>
       <c r="N29" s="52" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="48">
       <c r="A30" s="56" t="inlineStr">
         <is>
-          <t>ENGINE MOUNT AND LANDING GEAR MOUNT SERVICE LIFE</t>
+          <t>STRUCTURE SERVICE LIFE</t>
         </is>
       </c>
       <c r="B30" s="51" t="n"/>
@@ -4633,9 +4820,9 @@
     <row r="33" ht="15.75" customHeight="1" s="48">
       <c r="A33" s="25" t="n"/>
       <c r="B33" s="25" t="n"/>
-      <c r="C33" s="25" t="n"/>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="25" t="n"/>
+      <c r="C33" s="26" t="n"/>
+      <c r="D33" s="26" t="n"/>
+      <c r="E33" s="26" t="n"/>
       <c r="F33" s="25" t="n"/>
       <c r="G33" s="25" t="n"/>
       <c r="H33" s="25" t="n"/>
@@ -4649,9 +4836,9 @@
     <row r="34" ht="15.75" customHeight="1" s="48">
       <c r="A34" s="25" t="n"/>
       <c r="B34" s="25" t="n"/>
-      <c r="C34" s="25" t="n"/>
-      <c r="D34" s="25" t="n"/>
-      <c r="E34" s="25" t="n"/>
+      <c r="C34" s="26" t="n"/>
+      <c r="D34" s="26" t="n"/>
+      <c r="E34" s="26" t="n"/>
       <c r="F34" s="25" t="n"/>
       <c r="G34" s="25" t="n"/>
       <c r="H34" s="25" t="n"/>
@@ -4663,27 +4850,31 @@
       <c r="N34" s="52" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="48">
-      <c r="A35" s="25" t="n"/>
-      <c r="B35" s="25" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="25" t="n"/>
-      <c r="G35" s="25" t="n"/>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
-      <c r="J35" s="25" t="n"/>
-      <c r="K35" s="25" t="n"/>
-      <c r="L35" s="25" t="n"/>
-      <c r="M35" s="26" t="n"/>
+      <c r="A35" s="56" t="inlineStr">
+        <is>
+          <t>ENGINE MOUNT AND LANDING GEAR MOUNT SERVICE LIFE</t>
+        </is>
+      </c>
+      <c r="B35" s="51" t="n"/>
+      <c r="C35" s="51" t="n"/>
+      <c r="D35" s="51" t="n"/>
+      <c r="E35" s="51" t="n"/>
+      <c r="F35" s="51" t="n"/>
+      <c r="G35" s="51" t="n"/>
+      <c r="H35" s="51" t="n"/>
+      <c r="I35" s="51" t="n"/>
+      <c r="J35" s="51" t="n"/>
+      <c r="K35" s="51" t="n"/>
+      <c r="L35" s="51" t="n"/>
+      <c r="M35" s="51" t="n"/>
       <c r="N35" s="52" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="48">
       <c r="A36" s="25" t="n"/>
       <c r="B36" s="25" t="n"/>
-      <c r="C36" s="25" t="n"/>
-      <c r="D36" s="25" t="n"/>
-      <c r="E36" s="25" t="n"/>
+      <c r="C36" s="26" t="n"/>
+      <c r="D36" s="26" t="n"/>
+      <c r="E36" s="26" t="n"/>
       <c r="F36" s="25" t="n"/>
       <c r="G36" s="25" t="n"/>
       <c r="H36" s="25" t="n"/>
@@ -4697,9 +4888,9 @@
     <row r="37" ht="15.75" customHeight="1" s="48">
       <c r="A37" s="25" t="n"/>
       <c r="B37" s="25" t="n"/>
-      <c r="C37" s="25" t="n"/>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="25" t="n"/>
+      <c r="C37" s="26" t="n"/>
+      <c r="D37" s="26" t="n"/>
+      <c r="E37" s="26" t="n"/>
       <c r="F37" s="25" t="n"/>
       <c r="G37" s="25" t="n"/>
       <c r="H37" s="25" t="n"/>
@@ -4710,11 +4901,86 @@
       <c r="M37" s="26" t="n"/>
       <c r="N37" s="52" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="48"/>
-    <row r="39" ht="15.75" customHeight="1" s="48"/>
-    <row r="40" ht="15.75" customHeight="1" s="48"/>
-    <row r="41" ht="15.75" customHeight="1" s="48"/>
-    <row r="42" ht="15.75" customHeight="1" s="48"/>
+    <row r="38" ht="15.75" customHeight="1" s="48">
+      <c r="A38" s="25" t="n"/>
+      <c r="B38" s="25" t="n"/>
+      <c r="C38" s="25" t="n"/>
+      <c r="D38" s="25" t="n"/>
+      <c r="E38" s="25" t="n"/>
+      <c r="F38" s="25" t="n"/>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="25" t="n"/>
+      <c r="J38" s="25" t="n"/>
+      <c r="K38" s="25" t="n"/>
+      <c r="L38" s="25" t="n"/>
+      <c r="M38" s="26" t="n"/>
+      <c r="N38" s="52" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="48">
+      <c r="A39" s="25" t="n"/>
+      <c r="B39" s="25" t="n"/>
+      <c r="C39" s="25" t="n"/>
+      <c r="D39" s="25" t="n"/>
+      <c r="E39" s="25" t="n"/>
+      <c r="F39" s="25" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
+      <c r="J39" s="25" t="n"/>
+      <c r="K39" s="25" t="n"/>
+      <c r="L39" s="25" t="n"/>
+      <c r="M39" s="26" t="n"/>
+      <c r="N39" s="52" t="n"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="48">
+      <c r="A40" s="25" t="n"/>
+      <c r="B40" s="25" t="n"/>
+      <c r="C40" s="25" t="n"/>
+      <c r="D40" s="25" t="n"/>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="25" t="n"/>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
+      <c r="J40" s="25" t="n"/>
+      <c r="K40" s="25" t="n"/>
+      <c r="L40" s="25" t="n"/>
+      <c r="M40" s="26" t="n"/>
+      <c r="N40" s="52" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="48">
+      <c r="A41" s="25" t="n"/>
+      <c r="B41" s="25" t="n"/>
+      <c r="C41" s="25" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="25" t="n"/>
+      <c r="L41" s="25" t="n"/>
+      <c r="M41" s="26" t="n"/>
+      <c r="N41" s="52" t="n"/>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="48">
+      <c r="A42" s="25" t="n"/>
+      <c r="B42" s="25" t="n"/>
+      <c r="C42" s="25" t="n"/>
+      <c r="D42" s="25" t="n"/>
+      <c r="E42" s="25" t="n"/>
+      <c r="F42" s="25" t="n"/>
+      <c r="G42" s="25" t="n"/>
+      <c r="H42" s="25" t="n"/>
+      <c r="I42" s="25" t="n"/>
+      <c r="J42" s="25" t="n"/>
+      <c r="K42" s="25" t="n"/>
+      <c r="L42" s="25" t="n"/>
+      <c r="M42" s="26" t="n"/>
+      <c r="N42" s="52" t="n"/>
+    </row>
     <row r="43" ht="15.75" customHeight="1" s="48"/>
     <row r="44" ht="15.75" customHeight="1" s="48"/>
     <row r="45" ht="15.75" customHeight="1" s="48"/>

</xml_diff>

<commit_message>
Add aircraft AD applicability analysis
</commit_message>
<xml_diff>
--- a/Control_de_aeronavegabilidad2026.xlsx
+++ b/Control_de_aeronavegabilidad2026.xlsx
@@ -4528,100 +4528,76 @@
       <c r="N19" s="52" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="0" t="inlineStr">
         <is>
           <t>Access door latches</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="0" t="inlineStr">
         <is>
           <t>TB10 25012102</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="0" t="n">
         <v>1500</v>
       </c>
-      <c r="L20" t="inlineStr">
+      <c r="L20" s="0" t="inlineStr">
         <is>
           <t>Discard</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr">
+      <c r="M20" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB10 MM Rev.18 05-10-00 p.3</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="48">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="0" t="inlineStr">
         <is>
           <t>Teflon hoses</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="0" t="inlineStr">
         <is>
           <t>Teflon hoses</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L21" s="0" t="inlineStr">
         <is>
           <t>On Condition</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M21" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB10 MM Rev.18 05-10-00 p.5-9</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="48">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>Fuel selector filter/drain hose</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>TB10 52035114</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2000</v>
-      </c>
-      <c r="E22" t="n">
-        <v>3650</v>
-      </c>
-      <c r="L22" t="inlineStr">
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="48">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>Elastomer/rubber/vinyl hoses</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
+        <is>
+          <t>Assorted</t>
+        </is>
+      </c>
+      <c r="L23" s="0" t="inlineStr">
         <is>
           <t>Discard</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>SOCATA TB10 MM Rev.18 05-10-00 p.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="48">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Elastomer/rubber/vinyl hoses</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Assorted</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>3650</v>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Discard</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
+      <c r="M23" s="0" t="inlineStr">
         <is>
           <t>SOCATA TB10 MM Rev.18 05-10-00 p.5-9</t>
         </is>
@@ -4630,18 +4606,18 @@
     <row r="24" ht="15.75" customHeight="1" s="48"/>
     <row r="25" ht="15.75" customHeight="1" s="48">
       <c r="A25" s="25" t="n"/>
-      <c r="B25" s="25" t="n"/>
-      <c r="C25" s="25" t="n"/>
-      <c r="D25" s="25" t="n"/>
-      <c r="E25" s="25" t="n"/>
-      <c r="F25" s="25" t="n"/>
-      <c r="G25" s="25" t="n"/>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
-      <c r="J25" s="25" t="n"/>
-      <c r="K25" s="25" t="n"/>
-      <c r="L25" s="25" t="n"/>
-      <c r="M25" s="26" t="n"/>
+      <c r="B25" s="51" t="n"/>
+      <c r="C25" s="51" t="n"/>
+      <c r="D25" s="51" t="n"/>
+      <c r="E25" s="51" t="n"/>
+      <c r="F25" s="51" t="n"/>
+      <c r="G25" s="51" t="n"/>
+      <c r="H25" s="51" t="n"/>
+      <c r="I25" s="51" t="n"/>
+      <c r="J25" s="51" t="n"/>
+      <c r="K25" s="51" t="n"/>
+      <c r="L25" s="51" t="n"/>
+      <c r="M25" s="51" t="n"/>
       <c r="N25" s="52" t="n"/>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="48"/>
@@ -4662,7 +4638,7 @@
       <c r="J27" s="51" t="n"/>
       <c r="K27" s="51" t="n"/>
       <c r="L27" s="51" t="n"/>
-      <c r="M27" s="51" t="n"/>
+      <c r="M27" s="52" t="n"/>
       <c r="N27" s="52" t="n"/>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="48">
@@ -4786,9 +4762,19 @@
       <c r="N30" s="52" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="48">
-      <c r="A31" s="25" t="n"/>
-      <c r="B31" s="25" t="n"/>
-      <c r="C31" s="26" t="n"/>
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>Engine and Nose Landing Gear mounts</t>
+        </is>
+      </c>
+      <c r="B31" s="25" t="inlineStr">
+        <is>
+          <t>TB9/TB10/TB200 mounts</t>
+        </is>
+      </c>
+      <c r="C31" s="26" t="n">
+        <v>10000</v>
+      </c>
       <c r="D31" s="26" t="n"/>
       <c r="E31" s="26" t="n"/>
       <c r="F31" s="25" t="n"/>
@@ -4797,8 +4783,16 @@
       <c r="I31" s="25" t="n"/>
       <c r="J31" s="25" t="n"/>
       <c r="K31" s="25" t="n"/>
-      <c r="L31" s="25" t="n"/>
-      <c r="M31" s="26" t="n"/>
+      <c r="L31" s="25" t="inlineStr">
+        <is>
+          <t>Discard / Airworthiness Limitation</t>
+        </is>
+      </c>
+      <c r="M31" s="26" t="inlineStr">
+        <is>
+          <t>EASA AD 2007-0034; AMM Rev.18 ALS/time limits</t>
+        </is>
+      </c>
       <c r="N31" s="52" t="n"/>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="48">
@@ -4866,7 +4860,7 @@
       <c r="J35" s="51" t="n"/>
       <c r="K35" s="51" t="n"/>
       <c r="L35" s="51" t="n"/>
-      <c r="M35" s="51" t="n"/>
+      <c r="M35" s="52" t="n"/>
       <c r="N35" s="52" t="n"/>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="48">
@@ -5991,7 +5985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15.43" customWidth="1" style="48" min="1" max="1"/>
@@ -6221,17 +6215,17 @@
     <row r="9">
       <c r="A9" s="44" t="inlineStr">
         <is>
-          <t>2001-23-04</t>
+          <t>EASA 2007-0034</t>
         </is>
       </c>
       <c r="B9" s="44" t="inlineStr">
         <is>
-          <t>FAA</t>
+          <t>EASA</t>
         </is>
       </c>
       <c r="C9" s="44" t="inlineStr">
         <is>
-          <t>Fuel System</t>
+          <t>Time Limits - engine and NLG mounts</t>
         </is>
       </c>
       <c r="D9" s="26" t="n"/>
@@ -6245,7 +6239,7 @@
       <c r="L9" s="25" t="n"/>
       <c r="M9" s="45" t="inlineStr">
         <is>
-          <t>N/A por no sufrir impacto la hélice</t>
+          <t>Applicable. Introduces 10000 FH life limit; controlled in Life Limit/ALI.</t>
         </is>
       </c>
     </row>
@@ -6260,14 +6254,16 @@
           <t>EASA</t>
         </is>
       </c>
-      <c r="C10" s="44" t="n"/>
+      <c r="C10" s="44" t="inlineStr">
+        <is>
+          <t>Cabin access door hooks</t>
+        </is>
+      </c>
       <c r="D10" s="26" t="n">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="E10" s="26" t="n"/>
-      <c r="F10" s="26" t="n">
-        <v>180</v>
-      </c>
+      <c r="F10" s="26" t="n"/>
       <c r="G10" s="25" t="n"/>
       <c r="H10" s="25" t="n"/>
       <c r="I10" s="25" t="n"/>
@@ -6276,31 +6272,65 @@
       <c r="L10" s="25" t="n"/>
       <c r="M10" s="45" t="inlineStr">
         <is>
-          <t>N/A por número de serie</t>
+          <t>Uncertain: applies if aluminium/AU4G cabin access door hooks installed. Repetitive until terminating action.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="n"/>
-      <c r="B11" s="25" t="n"/>
-      <c r="C11" s="25" t="n"/>
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>EASA 2015-0130</t>
+        </is>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>EASA</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>Horizontal stabilizer spar inspection</t>
+        </is>
+      </c>
       <c r="D11" s="26" t="n"/>
       <c r="E11" s="26" t="n"/>
-      <c r="F11" s="26" t="n"/>
+      <c r="F11" s="26" t="n">
+        <v>2190</v>
+      </c>
       <c r="G11" s="25" t="n"/>
       <c r="H11" s="25" t="n"/>
       <c r="I11" s="25" t="n"/>
       <c r="J11" s="25" t="n"/>
       <c r="K11" s="25" t="n"/>
       <c r="L11" s="25" t="n"/>
-      <c r="M11" s="26" t="n"/>
+      <c r="M11" s="26" t="inlineStr">
+        <is>
+          <t>Applicable to all TB10 S/N. Repetitive 72 months.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="25" t="n"/>
-      <c r="B12" s="25" t="n"/>
-      <c r="C12" s="25" t="n"/>
-      <c r="D12" s="26" t="n"/>
-      <c r="E12" s="26" t="n"/>
+      <c r="A12" s="25" t="inlineStr">
+        <is>
+          <t>EASA 2018-0030R1</t>
+        </is>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>EASA</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Wing front attachments inspection/modification</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E12" s="26" t="n">
+        <v>3000</v>
+      </c>
       <c r="F12" s="26" t="n"/>
       <c r="G12" s="25" t="n"/>
       <c r="H12" s="25" t="n"/>
@@ -6308,27 +6338,61 @@
       <c r="J12" s="25" t="n"/>
       <c r="K12" s="25" t="n"/>
       <c r="L12" s="25" t="n"/>
-      <c r="M12" s="26" t="n"/>
+      <c r="M12" s="26" t="inlineStr">
+        <is>
+          <t>Applicable Group 1: TB10 MSN 001-803 includes S/N 649. Repetitive 2000 FH/3000 LDG; other actions per AD.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="25" t="n"/>
-      <c r="B13" s="25" t="n"/>
-      <c r="C13" s="25" t="n"/>
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>EASA 2025-0160</t>
+        </is>
+      </c>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>EASA</t>
+        </is>
+      </c>
+      <c r="C13" s="25" t="inlineStr">
+        <is>
+          <t>Lower rudder hinge fitting inspection</t>
+        </is>
+      </c>
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
-      <c r="F13" s="26" t="n"/>
+      <c r="F13" s="26" t="n">
+        <v>365</v>
+      </c>
       <c r="G13" s="25" t="n"/>
       <c r="H13" s="25" t="n"/>
       <c r="I13" s="25" t="n"/>
       <c r="J13" s="25" t="n"/>
       <c r="K13" s="25" t="n"/>
       <c r="L13" s="25" t="n"/>
-      <c r="M13" s="26" t="n"/>
+      <c r="M13" s="26" t="inlineStr">
+        <is>
+          <t>Applicable to all TB10 S/N. Repetitive 12 months.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="n"/>
-      <c r="B14" s="25" t="n"/>
-      <c r="C14" s="25" t="n"/>
+      <c r="A14" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-1992-206R3</t>
+        </is>
+      </c>
+      <c r="B14" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>Exhaust system</t>
+        </is>
+      </c>
       <c r="D14" s="26" t="n"/>
       <c r="E14" s="26" t="n"/>
       <c r="F14" s="26" t="n"/>
@@ -6338,12 +6402,28 @@
       <c r="J14" s="25" t="n"/>
       <c r="K14" s="25" t="n"/>
       <c r="L14" s="25" t="n"/>
-      <c r="M14" s="26" t="n"/>
+      <c r="M14" s="26" t="inlineStr">
+        <is>
+          <t>Applicable by S/N 1-1191; no repetitive requirement identified.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="25" t="n"/>
-      <c r="B15" s="25" t="n"/>
-      <c r="C15" s="25" t="n"/>
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-1994-264R1</t>
+        </is>
+      </c>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="inlineStr">
+        <is>
+          <t>Wing front attachments</t>
+        </is>
+      </c>
       <c r="D15" s="26" t="n"/>
       <c r="E15" s="26" t="n"/>
       <c r="F15" s="26" t="n"/>
@@ -6353,14 +6433,34 @@
       <c r="J15" s="25" t="n"/>
       <c r="K15" s="25" t="n"/>
       <c r="L15" s="25" t="n"/>
-      <c r="M15" s="26" t="n"/>
+      <c r="M15" s="26" t="inlineStr">
+        <is>
+          <t>N/A: superseded by EASA 2018-0030R1.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="n"/>
-      <c r="B16" s="25" t="n"/>
-      <c r="C16" s="25" t="n"/>
-      <c r="D16" s="26" t="n"/>
-      <c r="E16" s="26" t="n"/>
+      <c r="A16" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-1994-265R4</t>
+        </is>
+      </c>
+      <c r="B16" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>Main landing gear support ribs</t>
+        </is>
+      </c>
+      <c r="D16" s="26" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>1500</v>
+      </c>
       <c r="F16" s="26" t="n"/>
       <c r="G16" s="25" t="n"/>
       <c r="H16" s="25" t="n"/>
@@ -6368,12 +6468,28 @@
       <c r="J16" s="25" t="n"/>
       <c r="K16" s="25" t="n"/>
       <c r="L16" s="25" t="n"/>
-      <c r="M16" s="26" t="n"/>
+      <c r="M16" s="26" t="inlineStr">
+        <is>
+          <t>Applicable/conditional Case A for TB10 S/N 1-803; repetitive 1000 FH/1500 LDG unless reinforced/kit case applies.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="25" t="n"/>
-      <c r="B17" s="25" t="n"/>
-      <c r="C17" s="25" t="n"/>
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-1996-143</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="inlineStr">
+        <is>
+          <t>Front belt upper attachment</t>
+        </is>
+      </c>
       <c r="D17" s="25" t="n"/>
       <c r="E17" s="25" t="n"/>
       <c r="F17" s="25" t="n"/>
@@ -6383,12 +6499,28 @@
       <c r="J17" s="25" t="n"/>
       <c r="K17" s="25" t="n"/>
       <c r="L17" s="25" t="n"/>
-      <c r="M17" s="26" t="n"/>
+      <c r="M17" s="26" t="inlineStr">
+        <is>
+          <t>Uncertain: S/N range includes 649 but depends on upholstering on upper duct posts.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="n"/>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-1999-062</t>
+        </is>
+      </c>
+      <c r="B18" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="inlineStr">
+        <is>
+          <t>Fuel system / 14V fuel gauge placard</t>
+        </is>
+      </c>
       <c r="D18" s="25" t="n"/>
       <c r="E18" s="25" t="n"/>
       <c r="F18" s="25" t="n"/>
@@ -6398,12 +6530,28 @@
       <c r="J18" s="25" t="n"/>
       <c r="K18" s="25" t="n"/>
       <c r="L18" s="25" t="n"/>
-      <c r="M18" s="26" t="n"/>
+      <c r="M18" s="26" t="inlineStr">
+        <is>
+          <t>Uncertain: S/N 649 in 14V range; depends on engine control panel amendment D.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="25" t="n"/>
-      <c r="B19" s="25" t="n"/>
-      <c r="C19" s="25" t="n"/>
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-002</t>
+        </is>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="inlineStr">
+        <is>
+          <t>Rudder bearing</t>
+        </is>
+      </c>
       <c r="D19" s="25" t="n"/>
       <c r="E19" s="25" t="n"/>
       <c r="F19" s="25" t="n"/>
@@ -6413,12 +6561,28 @@
       <c r="J19" s="25" t="n"/>
       <c r="K19" s="25" t="n"/>
       <c r="L19" s="25" t="n"/>
-      <c r="M19" s="26" t="n"/>
+      <c r="M19" s="26" t="inlineStr">
+        <is>
+          <t>N/A: superseded by EASA 2025-0160.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="25" t="n"/>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="25" t="n"/>
+      <c r="A20" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-005</t>
+        </is>
+      </c>
+      <c r="B20" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="inlineStr">
+        <is>
+          <t>Seat unlocking</t>
+        </is>
+      </c>
       <c r="D20" s="25" t="n"/>
       <c r="E20" s="25" t="n"/>
       <c r="F20" s="25" t="n"/>
@@ -6428,12 +6592,28 @@
       <c r="J20" s="25" t="n"/>
       <c r="K20" s="25" t="n"/>
       <c r="L20" s="25" t="n"/>
-      <c r="M20" s="26" t="n"/>
+      <c r="M20" s="26" t="inlineStr">
+        <is>
+          <t>Uncertain: applies unless MOD 165 embodied in production.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="48">
-      <c r="A21" s="25" t="n"/>
-      <c r="B21" s="25" t="n"/>
-      <c r="C21" s="25" t="n"/>
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-305</t>
+        </is>
+      </c>
+      <c r="B21" s="25" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="inlineStr">
+        <is>
+          <t>Nose gear fork spare part</t>
+        </is>
+      </c>
       <c r="D21" s="25" t="n"/>
       <c r="E21" s="25" t="n"/>
       <c r="F21" s="25" t="n"/>
@@ -6443,213 +6623,218 @@
       <c r="J21" s="25" t="n"/>
       <c r="K21" s="25" t="n"/>
       <c r="L21" s="25" t="n"/>
-      <c r="M21" s="26" t="n"/>
+      <c r="M21" s="26" t="inlineStr">
+        <is>
+          <t>Uncertain: only if affected spare fork installed.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="48">
-      <c r="A22" s="59" t="inlineStr">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-306</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Wing front attaching bolts</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Uncertain/N/A by S/N: S/N 649 not listed; applies only if affected spare axes installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="48">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-446R1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Ammeter circuit option</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on ammeter option OPT 10 593/689/D689 installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="48">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DGAC F-2003-368R2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DGAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Aileron/elevator gimbal joints</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>110</v>
+      </c>
+      <c r="F24" t="n">
+        <v>420</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Uncertain: applies unless MOD 10-0209-27 or terminating SB action embodied; repetitive 110 FH/14 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="48"/>
+    <row r="26" ht="15.75" customHeight="1" s="48">
+      <c r="A26" s="59" t="inlineStr">
         <is>
           <t>Engine</t>
         </is>
       </c>
-      <c r="B22" s="51" t="n"/>
-      <c r="C22" s="51" t="n"/>
-      <c r="D22" s="51" t="n"/>
-      <c r="E22" s="51" t="n"/>
-      <c r="F22" s="51" t="n"/>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="51" t="n"/>
-      <c r="I22" s="51" t="n"/>
-      <c r="J22" s="51" t="n"/>
-      <c r="K22" s="51" t="n"/>
-      <c r="L22" s="51" t="n"/>
-      <c r="M22" s="52" t="n"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="48">
-      <c r="A23" s="13" t="n"/>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="18" t="inlineStr">
+      <c r="B26" s="51" t="n"/>
+      <c r="C26" s="51" t="n"/>
+      <c r="D26" s="51" t="n"/>
+      <c r="E26" s="51" t="n"/>
+      <c r="F26" s="51" t="n"/>
+      <c r="G26" s="51" t="n"/>
+      <c r="H26" s="51" t="n"/>
+      <c r="I26" s="51" t="n"/>
+      <c r="J26" s="51" t="n"/>
+      <c r="K26" s="51" t="n"/>
+      <c r="L26" s="51" t="n"/>
+      <c r="M26" s="52" t="n"/>
+    </row>
+    <row r="27" ht="15.75" customHeight="1" s="48">
+      <c r="A27" s="13" t="n"/>
+      <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="18" t="inlineStr">
         <is>
           <t>Interval /TBO</t>
         </is>
       </c>
-      <c r="E23" s="51" t="n"/>
-      <c r="F23" s="52" t="n"/>
-      <c r="G23" s="47" t="inlineStr">
+      <c r="E27" s="51" t="n"/>
+      <c r="F27" s="52" t="n"/>
+      <c r="G27" s="47" t="inlineStr">
         <is>
           <t>Interval FH/ CyC/Ldgs</t>
         </is>
       </c>
-      <c r="H23" s="51" t="n"/>
-      <c r="I23" s="52" t="n"/>
-      <c r="J23" s="47" t="inlineStr">
+      <c r="H27" s="51" t="n"/>
+      <c r="I27" s="52" t="n"/>
+      <c r="J27" s="47" t="inlineStr">
         <is>
           <t>Calendar</t>
         </is>
       </c>
-      <c r="K23" s="51" t="n"/>
-      <c r="L23" s="52" t="n"/>
-      <c r="M23" s="47" t="inlineStr">
+      <c r="K27" s="51" t="n"/>
+      <c r="L27" s="52" t="n"/>
+      <c r="M27" s="47" t="inlineStr">
         <is>
           <t>Applicable ICA reference</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="48">
-      <c r="A24" s="18" t="inlineStr">
+    <row r="28" ht="15.75" customHeight="1" s="48">
+      <c r="A28" s="18" t="inlineStr">
         <is>
           <t>AD Number</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>NAA</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C28" s="18" t="inlineStr">
         <is>
           <t>Subject</t>
         </is>
       </c>
-      <c r="D24" s="39" t="inlineStr">
+      <c r="D28" s="39" t="inlineStr">
         <is>
           <t>FH</t>
         </is>
       </c>
-      <c r="E24" s="40" t="inlineStr">
+      <c r="E28" s="40" t="inlineStr">
         <is>
           <t>Ldg/Cycle</t>
         </is>
       </c>
-      <c r="F24" s="40" t="inlineStr">
+      <c r="F28" s="40" t="inlineStr">
         <is>
           <t>days</t>
         </is>
       </c>
-      <c r="G24" s="41" t="inlineStr">
+      <c r="G28" s="41" t="inlineStr">
         <is>
           <t>Performed</t>
         </is>
       </c>
-      <c r="H24" s="42" t="inlineStr">
+      <c r="H28" s="42" t="inlineStr">
         <is>
           <t>Next due</t>
         </is>
       </c>
-      <c r="I24" s="43" t="inlineStr">
+      <c r="I28" s="43" t="inlineStr">
         <is>
           <t>to go</t>
         </is>
       </c>
-      <c r="J24" s="41" t="inlineStr">
+      <c r="J28" s="41" t="inlineStr">
         <is>
           <t>Performed</t>
         </is>
       </c>
-      <c r="K24" s="42" t="inlineStr">
+      <c r="K28" s="42" t="inlineStr">
         <is>
           <t>Next due</t>
         </is>
       </c>
-      <c r="L24" s="43" t="inlineStr">
+      <c r="L28" s="43" t="inlineStr">
         <is>
           <t>to go</t>
         </is>
       </c>
-      <c r="M24" s="26" t="inlineStr">
+      <c r="M28" s="26" t="inlineStr">
         <is>
           <t>Remarcks</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1" s="48">
-      <c r="A25" s="44" t="inlineStr">
+    <row r="29" ht="15.75" customHeight="1" s="48">
+      <c r="A29" s="44" t="inlineStr">
         <is>
           <t>2001-23-04</t>
         </is>
       </c>
-      <c r="B25" s="44" t="inlineStr">
+      <c r="B29" s="44" t="inlineStr">
         <is>
           <t>FAA</t>
         </is>
       </c>
-      <c r="C25" s="44" t="inlineStr">
+      <c r="C29" s="44" t="inlineStr">
         <is>
           <t>Fuel System</t>
         </is>
       </c>
-      <c r="D25" s="26" t="n"/>
-      <c r="E25" s="26" t="n"/>
-      <c r="F25" s="26" t="n"/>
-      <c r="G25" s="25" t="n"/>
-      <c r="H25" s="25" t="n"/>
-      <c r="I25" s="25" t="n"/>
-      <c r="J25" s="25" t="n"/>
-      <c r="K25" s="25" t="n"/>
-      <c r="L25" s="25" t="n"/>
-      <c r="M25" s="45" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="48">
-      <c r="A26" s="44" t="inlineStr">
-        <is>
-          <t>EASA 2007-0101</t>
-        </is>
-      </c>
-      <c r="B26" s="44" t="inlineStr">
-        <is>
-          <t>EASA</t>
-        </is>
-      </c>
-      <c r="C26" s="44" t="n"/>
-      <c r="D26" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="E26" s="26" t="n"/>
-      <c r="F26" s="26" t="n">
-        <v>180</v>
-      </c>
-      <c r="G26" s="25" t="n"/>
-      <c r="H26" s="25" t="n"/>
-      <c r="I26" s="25" t="n"/>
-      <c r="J26" s="25" t="n"/>
-      <c r="K26" s="25" t="n"/>
-      <c r="L26" s="25" t="n"/>
-      <c r="M26" s="45" t="n"/>
-    </row>
-    <row r="27" ht="15.75" customHeight="1" s="48">
-      <c r="A27" s="25" t="n"/>
-      <c r="B27" s="25" t="n"/>
-      <c r="C27" s="25" t="n"/>
-      <c r="D27" s="26" t="n"/>
-      <c r="E27" s="26" t="n"/>
-      <c r="F27" s="26" t="n"/>
-      <c r="G27" s="25" t="n"/>
-      <c r="H27" s="25" t="n"/>
-      <c r="I27" s="25" t="n"/>
-      <c r="J27" s="25" t="n"/>
-      <c r="K27" s="25" t="n"/>
-      <c r="L27" s="25" t="n"/>
-      <c r="M27" s="26" t="n"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" s="48">
-      <c r="A28" s="25" t="n"/>
-      <c r="B28" s="25" t="n"/>
-      <c r="C28" s="25" t="n"/>
-      <c r="D28" s="26" t="n"/>
-      <c r="E28" s="26" t="n"/>
-      <c r="F28" s="26" t="n"/>
-      <c r="G28" s="25" t="n"/>
-      <c r="H28" s="25" t="n"/>
-      <c r="I28" s="25" t="n"/>
-      <c r="J28" s="25" t="n"/>
-      <c r="K28" s="25" t="n"/>
-      <c r="L28" s="25" t="n"/>
-      <c r="M28" s="26" t="n"/>
-    </row>
-    <row r="29" ht="15.75" customHeight="1" s="48">
-      <c r="A29" s="25" t="n"/>
-      <c r="B29" s="25" t="n"/>
-      <c r="C29" s="25" t="n"/>
       <c r="D29" s="26" t="n"/>
       <c r="E29" s="26" t="n"/>
       <c r="F29" s="26" t="n"/>
@@ -6659,22 +6844,34 @@
       <c r="J29" s="25" t="n"/>
       <c r="K29" s="25" t="n"/>
       <c r="L29" s="25" t="n"/>
-      <c r="M29" s="26" t="n"/>
+      <c r="M29" s="45" t="n"/>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="48">
-      <c r="A30" s="25" t="n"/>
-      <c r="B30" s="25" t="n"/>
-      <c r="C30" s="25" t="n"/>
-      <c r="D30" s="26" t="n"/>
+      <c r="A30" s="44" t="inlineStr">
+        <is>
+          <t>EASA 2007-0101</t>
+        </is>
+      </c>
+      <c r="B30" s="44" t="inlineStr">
+        <is>
+          <t>EASA</t>
+        </is>
+      </c>
+      <c r="C30" s="44" t="n"/>
+      <c r="D30" s="26" t="n">
+        <v>100</v>
+      </c>
       <c r="E30" s="26" t="n"/>
-      <c r="F30" s="26" t="n"/>
+      <c r="F30" s="26" t="n">
+        <v>180</v>
+      </c>
       <c r="G30" s="25" t="n"/>
       <c r="H30" s="25" t="n"/>
       <c r="I30" s="25" t="n"/>
       <c r="J30" s="25" t="n"/>
       <c r="K30" s="25" t="n"/>
       <c r="L30" s="25" t="n"/>
-      <c r="M30" s="26" t="n"/>
+      <c r="M30" s="45" t="n"/>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="48">
       <c r="A31" s="25" t="n"/>
@@ -6710,9 +6907,9 @@
       <c r="A33" s="25" t="n"/>
       <c r="B33" s="25" t="n"/>
       <c r="C33" s="25" t="n"/>
-      <c r="D33" s="25" t="n"/>
-      <c r="E33" s="25" t="n"/>
-      <c r="F33" s="25" t="n"/>
+      <c r="D33" s="26" t="n"/>
+      <c r="E33" s="26" t="n"/>
+      <c r="F33" s="26" t="n"/>
       <c r="G33" s="25" t="n"/>
       <c r="H33" s="25" t="n"/>
       <c r="I33" s="25" t="n"/>
@@ -6725,9 +6922,9 @@
       <c r="A34" s="25" t="n"/>
       <c r="B34" s="25" t="n"/>
       <c r="C34" s="25" t="n"/>
-      <c r="D34" s="25" t="n"/>
-      <c r="E34" s="25" t="n"/>
-      <c r="F34" s="25" t="n"/>
+      <c r="D34" s="26" t="n"/>
+      <c r="E34" s="26" t="n"/>
+      <c r="F34" s="26" t="n"/>
       <c r="G34" s="25" t="n"/>
       <c r="H34" s="25" t="n"/>
       <c r="I34" s="25" t="n"/>
@@ -6740,9 +6937,9 @@
       <c r="A35" s="25" t="n"/>
       <c r="B35" s="25" t="n"/>
       <c r="C35" s="25" t="n"/>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="25" t="n"/>
+      <c r="D35" s="26" t="n"/>
+      <c r="E35" s="26" t="n"/>
+      <c r="F35" s="26" t="n"/>
       <c r="G35" s="25" t="n"/>
       <c r="H35" s="25" t="n"/>
       <c r="I35" s="25" t="n"/>
@@ -6755,9 +6952,9 @@
       <c r="A36" s="25" t="n"/>
       <c r="B36" s="25" t="n"/>
       <c r="C36" s="25" t="n"/>
-      <c r="D36" s="25" t="n"/>
-      <c r="E36" s="25" t="n"/>
-      <c r="F36" s="25" t="n"/>
+      <c r="D36" s="26" t="n"/>
+      <c r="E36" s="26" t="n"/>
+      <c r="F36" s="26" t="n"/>
       <c r="G36" s="25" t="n"/>
       <c r="H36" s="25" t="n"/>
       <c r="I36" s="25" t="n"/>
@@ -6781,10 +6978,66 @@
       <c r="L37" s="25" t="n"/>
       <c r="M37" s="26" t="n"/>
     </row>
-    <row r="38" ht="15.75" customHeight="1" s="48"/>
-    <row r="39" ht="15.75" customHeight="1" s="48"/>
-    <row r="40" ht="15.75" customHeight="1" s="48"/>
-    <row r="41" ht="15.75" customHeight="1" s="48"/>
+    <row r="38" ht="15.75" customHeight="1" s="48">
+      <c r="A38" s="25" t="n"/>
+      <c r="B38" s="25" t="n"/>
+      <c r="C38" s="25" t="n"/>
+      <c r="D38" s="25" t="n"/>
+      <c r="E38" s="25" t="n"/>
+      <c r="F38" s="25" t="n"/>
+      <c r="G38" s="25" t="n"/>
+      <c r="H38" s="25" t="n"/>
+      <c r="I38" s="25" t="n"/>
+      <c r="J38" s="25" t="n"/>
+      <c r="K38" s="25" t="n"/>
+      <c r="L38" s="25" t="n"/>
+      <c r="M38" s="26" t="n"/>
+    </row>
+    <row r="39" ht="15.75" customHeight="1" s="48">
+      <c r="A39" s="25" t="n"/>
+      <c r="B39" s="25" t="n"/>
+      <c r="C39" s="25" t="n"/>
+      <c r="D39" s="25" t="n"/>
+      <c r="E39" s="25" t="n"/>
+      <c r="F39" s="25" t="n"/>
+      <c r="G39" s="25" t="n"/>
+      <c r="H39" s="25" t="n"/>
+      <c r="I39" s="25" t="n"/>
+      <c r="J39" s="25" t="n"/>
+      <c r="K39" s="25" t="n"/>
+      <c r="L39" s="25" t="n"/>
+      <c r="M39" s="26" t="n"/>
+    </row>
+    <row r="40" ht="15.75" customHeight="1" s="48">
+      <c r="A40" s="25" t="n"/>
+      <c r="B40" s="25" t="n"/>
+      <c r="C40" s="25" t="n"/>
+      <c r="D40" s="25" t="n"/>
+      <c r="E40" s="25" t="n"/>
+      <c r="F40" s="25" t="n"/>
+      <c r="G40" s="25" t="n"/>
+      <c r="H40" s="25" t="n"/>
+      <c r="I40" s="25" t="n"/>
+      <c r="J40" s="25" t="n"/>
+      <c r="K40" s="25" t="n"/>
+      <c r="L40" s="25" t="n"/>
+      <c r="M40" s="26" t="n"/>
+    </row>
+    <row r="41" ht="15.75" customHeight="1" s="48">
+      <c r="A41" s="25" t="n"/>
+      <c r="B41" s="25" t="n"/>
+      <c r="C41" s="25" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="25" t="n"/>
+      <c r="H41" s="25" t="n"/>
+      <c r="I41" s="25" t="n"/>
+      <c r="J41" s="25" t="n"/>
+      <c r="K41" s="25" t="n"/>
+      <c r="L41" s="25" t="n"/>
+      <c r="M41" s="26" t="n"/>
+    </row>
     <row r="42" ht="15.75" customHeight="1" s="48"/>
     <row r="43" ht="15.75" customHeight="1" s="48"/>
     <row r="44" ht="15.75" customHeight="1" s="48"/>

</xml_diff>

<commit_message>
Add engine AD applicability analysis
</commit_message>
<xml_diff>
--- a/Control_de_aeronavegabilidad2026.xlsx
+++ b/Control_de_aeronavegabilidad2026.xlsx
@@ -5985,7 +5985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="15.43" customWidth="1" style="48" min="1" max="1"/>
@@ -6630,72 +6630,57 @@
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="48">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="0" t="inlineStr">
         <is>
           <t>DGAC F-2001-306</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+    </row>
+    <row r="23" ht="15.75" customHeight="1" s="48">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>DGAC F-2001-446R1</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="inlineStr">
         <is>
           <t>DGAC</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Wing front attaching bolts</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Uncertain/N/A by S/N: S/N 649 not listed; applies only if affected spare axes installed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="48">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>DGAC F-2001-446R1</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
+        <is>
+          <t>Ammeter circuit option</t>
+        </is>
+      </c>
+      <c r="M23" s="0" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on ammeter option OPT 10 593/689/D689 installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="48">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>DGAC F-2003-368R2</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
         <is>
           <t>DGAC</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Ammeter circuit option</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Uncertain: depends on ammeter option OPT 10 593/689/D689 installed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="48">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>DGAC F-2003-368R2</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>DGAC</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>Aileron/elevator gimbal joints</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" s="0" t="n">
         <v>110</v>
       </c>
-      <c r="F24" t="n">
+      <c r="F24" s="0" t="n">
         <v>420</v>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M24" s="0" t="inlineStr">
         <is>
           <t>Uncertain: applies unless MOD 10-0209-27 or terminating SB action embodied; repetitive 110 FH/14 months.</t>
         </is>
@@ -6822,20 +6807,22 @@
     <row r="29" ht="15.75" customHeight="1" s="48">
       <c r="A29" s="44" t="inlineStr">
         <is>
-          <t>2001-23-04</t>
+          <t>EASA 2005-0023R3</t>
         </is>
       </c>
       <c r="B29" s="44" t="inlineStr">
         <is>
-          <t>FAA</t>
+          <t>EASA</t>
         </is>
       </c>
       <c r="C29" s="44" t="inlineStr">
         <is>
-          <t>Fuel System</t>
-        </is>
-      </c>
-      <c r="D29" s="26" t="n"/>
+          <t>Exhaust valve and guide inspection</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="n">
+        <v>440</v>
+      </c>
       <c r="E29" s="26" t="n"/>
       <c r="F29" s="26" t="n"/>
       <c r="G29" s="25" t="n"/>
@@ -6844,12 +6831,16 @@
       <c r="J29" s="25" t="n"/>
       <c r="K29" s="25" t="n"/>
       <c r="L29" s="25" t="n"/>
-      <c r="M29" s="45" t="n"/>
+      <c r="M29" s="45" t="inlineStr">
+        <is>
+          <t>Applicable: all Lycoming piston engines; repetitive if no Hi-Chrome guides.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="48">
       <c r="A30" s="44" t="inlineStr">
         <is>
-          <t>EASA 2007-0101</t>
+          <t>EASA 2024-0111</t>
         </is>
       </c>
       <c r="B30" s="44" t="inlineStr">
@@ -6857,208 +6848,662 @@
           <t>EASA</t>
         </is>
       </c>
-      <c r="C30" s="44" t="n"/>
-      <c r="D30" s="26" t="n">
-        <v>100</v>
-      </c>
+      <c r="C30" s="44" t="inlineStr">
+        <is>
+          <t>Reciprocating engine inspection</t>
+        </is>
+      </c>
+      <c r="D30" s="26" t="n"/>
       <c r="E30" s="26" t="n"/>
-      <c r="F30" s="26" t="n">
-        <v>180</v>
-      </c>
+      <c r="F30" s="26" t="n"/>
       <c r="G30" s="25" t="n"/>
       <c r="H30" s="25" t="n"/>
       <c r="I30" s="25" t="n"/>
       <c r="J30" s="25" t="n"/>
       <c r="K30" s="25" t="n"/>
       <c r="L30" s="25" t="n"/>
-      <c r="M30" s="45" t="n"/>
+      <c r="M30" s="45" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on manufacture/overhaul date and TCCA AD CF-2005-40 criteria.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="48">
-      <c r="A31" s="25" t="n"/>
-      <c r="B31" s="25" t="n"/>
-      <c r="C31" s="25" t="n"/>
-      <c r="D31" s="26" t="n"/>
-      <c r="E31" s="26" t="n"/>
-      <c r="F31" s="26" t="n"/>
-      <c r="G31" s="25" t="n"/>
-      <c r="H31" s="25" t="n"/>
-      <c r="I31" s="25" t="n"/>
-      <c r="J31" s="25" t="n"/>
-      <c r="K31" s="25" t="n"/>
-      <c r="L31" s="25" t="n"/>
-      <c r="M31" s="26" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>FAA 2002-12-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Oil filter converter plate gasket</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>50</v>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Uncertain: O-360-A1AD listed; applies by shipping date or affected gasket/kit until terminating action.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="48">
-      <c r="A32" s="25" t="n"/>
-      <c r="B32" s="25" t="n"/>
-      <c r="C32" s="25" t="n"/>
-      <c r="D32" s="26" t="n"/>
-      <c r="E32" s="26" t="n"/>
-      <c r="F32" s="26" t="n"/>
-      <c r="G32" s="25" t="n"/>
-      <c r="H32" s="25" t="n"/>
-      <c r="I32" s="25" t="n"/>
-      <c r="J32" s="25" t="n"/>
-      <c r="K32" s="25" t="n"/>
-      <c r="L32" s="25" t="n"/>
-      <c r="M32" s="26" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>FAA 2004-10-14</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Crankshaft gear retaining bolt</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Applicable only after propeller strike event; not repetitive.</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="48">
-      <c r="A33" s="25" t="n"/>
-      <c r="B33" s="25" t="n"/>
-      <c r="C33" s="25" t="n"/>
-      <c r="D33" s="26" t="n"/>
-      <c r="E33" s="26" t="n"/>
-      <c r="F33" s="26" t="n"/>
-      <c r="G33" s="25" t="n"/>
-      <c r="H33" s="25" t="n"/>
-      <c r="I33" s="25" t="n"/>
-      <c r="J33" s="25" t="n"/>
-      <c r="K33" s="25" t="n"/>
-      <c r="L33" s="25" t="n"/>
-      <c r="M33" s="26" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FAA 2005-19-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Crankshaft replacement</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on manufacture/rebuild/overhaul date or crankshaft installation.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="48">
-      <c r="A34" s="25" t="n"/>
-      <c r="B34" s="25" t="n"/>
-      <c r="C34" s="25" t="n"/>
-      <c r="D34" s="26" t="n"/>
-      <c r="E34" s="26" t="n"/>
-      <c r="F34" s="26" t="n"/>
-      <c r="G34" s="25" t="n"/>
-      <c r="H34" s="25" t="n"/>
-      <c r="I34" s="25" t="n"/>
-      <c r="J34" s="25" t="n"/>
-      <c r="K34" s="25" t="n"/>
-      <c r="L34" s="25" t="n"/>
-      <c r="M34" s="26" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>FAA 2005-26-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ECi Classic Cast cylinders</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on affected ECi cylinders installed.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="48">
-      <c r="A35" s="25" t="n"/>
-      <c r="B35" s="25" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="26" t="n"/>
-      <c r="E35" s="26" t="n"/>
-      <c r="F35" s="26" t="n"/>
-      <c r="G35" s="25" t="n"/>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
-      <c r="J35" s="25" t="n"/>
-      <c r="K35" s="25" t="n"/>
-      <c r="L35" s="25" t="n"/>
-      <c r="M35" s="26" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>FAA 2006-10-21</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>ECi connecting rods</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on affected ECi connecting rods installed.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="48">
-      <c r="A36" s="25" t="n"/>
-      <c r="B36" s="25" t="n"/>
-      <c r="C36" s="25" t="n"/>
-      <c r="D36" s="26" t="n"/>
-      <c r="E36" s="26" t="n"/>
-      <c r="F36" s="26" t="n"/>
-      <c r="G36" s="25" t="n"/>
-      <c r="H36" s="25" t="n"/>
-      <c r="I36" s="25" t="n"/>
-      <c r="J36" s="25" t="n"/>
-      <c r="K36" s="25" t="n"/>
-      <c r="L36" s="25" t="n"/>
-      <c r="M36" s="26" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>FAA 2006-12-07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ECi Classic Cast cylinders</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on affected ECi cylinders installed.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="48">
-      <c r="A37" s="25" t="n"/>
-      <c r="B37" s="25" t="n"/>
-      <c r="C37" s="25" t="n"/>
-      <c r="D37" s="25" t="n"/>
-      <c r="E37" s="25" t="n"/>
-      <c r="F37" s="25" t="n"/>
-      <c r="G37" s="25" t="n"/>
-      <c r="H37" s="25" t="n"/>
-      <c r="I37" s="25" t="n"/>
-      <c r="J37" s="25" t="n"/>
-      <c r="K37" s="25" t="n"/>
-      <c r="L37" s="25" t="n"/>
-      <c r="M37" s="26" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>FAA 2006-20-09</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Crankshaft replacement</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>Uncertain/superseded logic: depends on MSB listed engine/crankshaft S/N; see FAA 2012-19-01.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="48">
-      <c r="A38" s="25" t="n"/>
-      <c r="B38" s="25" t="n"/>
-      <c r="C38" s="25" t="n"/>
-      <c r="D38" s="25" t="n"/>
-      <c r="E38" s="25" t="n"/>
-      <c r="F38" s="25" t="n"/>
-      <c r="G38" s="25" t="n"/>
-      <c r="H38" s="25" t="n"/>
-      <c r="I38" s="25" t="n"/>
-      <c r="J38" s="25" t="n"/>
-      <c r="K38" s="25" t="n"/>
-      <c r="L38" s="25" t="n"/>
-      <c r="M38" s="26" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>FAA 2007-04-19R1</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Superior Air Parts cylinders</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on affected SAP cylinders installed.</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="48">
-      <c r="A39" s="25" t="n"/>
-      <c r="B39" s="25" t="n"/>
-      <c r="C39" s="25" t="n"/>
-      <c r="D39" s="25" t="n"/>
-      <c r="E39" s="25" t="n"/>
-      <c r="F39" s="25" t="n"/>
-      <c r="G39" s="25" t="n"/>
-      <c r="H39" s="25" t="n"/>
-      <c r="I39" s="25" t="n"/>
-      <c r="J39" s="25" t="n"/>
-      <c r="K39" s="25" t="n"/>
-      <c r="L39" s="25" t="n"/>
-      <c r="M39" s="26" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>FAA 2008-19-05</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ECi Titan cylinders</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>50</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Uncertain: O-360-A1AD listed; repetitive if affected ECi Titan cylinders installed.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="48">
-      <c r="A40" s="25" t="n"/>
-      <c r="B40" s="25" t="n"/>
-      <c r="C40" s="25" t="n"/>
-      <c r="D40" s="25" t="n"/>
-      <c r="E40" s="25" t="n"/>
-      <c r="F40" s="25" t="n"/>
-      <c r="G40" s="25" t="n"/>
-      <c r="H40" s="25" t="n"/>
-      <c r="I40" s="25" t="n"/>
-      <c r="J40" s="25" t="n"/>
-      <c r="K40" s="25" t="n"/>
-      <c r="L40" s="25" t="n"/>
-      <c r="M40" s="26" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>FAA 2009-26-12</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ECi Titan cylinders</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>50</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Uncertain: O-360-A1AD listed; repetitive if affected ECi Titan cylinders installed.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="48">
-      <c r="A41" s="25" t="n"/>
-      <c r="B41" s="25" t="n"/>
-      <c r="C41" s="25" t="n"/>
-      <c r="D41" s="25" t="n"/>
-      <c r="E41" s="25" t="n"/>
-      <c r="F41" s="25" t="n"/>
-      <c r="G41" s="25" t="n"/>
-      <c r="H41" s="25" t="n"/>
-      <c r="I41" s="25" t="n"/>
-      <c r="J41" s="25" t="n"/>
-      <c r="K41" s="25" t="n"/>
-      <c r="L41" s="25" t="n"/>
-      <c r="M41" s="26" t="n"/>
-    </row>
-    <row r="42" ht="15.75" customHeight="1" s="48"/>
-    <row r="43" ht="15.75" customHeight="1" s="48"/>
-    <row r="44" ht="15.75" customHeight="1" s="48"/>
-    <row r="45" ht="15.75" customHeight="1" s="48"/>
-    <row r="46" ht="15.75" customHeight="1" s="48"/>
-    <row r="47" ht="15.75" customHeight="1" s="48"/>
-    <row r="48" ht="15.75" customHeight="1" s="48"/>
-    <row r="49" ht="15.75" customHeight="1" s="48"/>
-    <row r="50" ht="15.75" customHeight="1" s="48"/>
-    <row r="51" ht="15.75" customHeight="1" s="48"/>
-    <row r="52" ht="15.75" customHeight="1" s="48"/>
-    <row r="53" ht="15.75" customHeight="1" s="48"/>
-    <row r="54" ht="15.75" customHeight="1" s="48"/>
-    <row r="55" ht="15.75" customHeight="1" s="48"/>
-    <row r="56" ht="15.75" customHeight="1" s="48"/>
-    <row r="57" ht="15.75" customHeight="1" s="48"/>
-    <row r="58" ht="15.75" customHeight="1" s="48"/>
-    <row r="59" ht="15.75" customHeight="1" s="48"/>
-    <row r="60" ht="15.75" customHeight="1" s="48"/>
-    <row r="61" ht="15.75" customHeight="1" s="48"/>
-    <row r="62" ht="15.75" customHeight="1" s="48"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>FAA 2010-07-08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>KAES rebuilt turbochargers</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>N/A: O-360-A1AD is naturally aspirated, no turbocharger.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1" s="48">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>FAA 2012-03-07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>HA-6 carburetor inspection/replacement</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Uncertain/N/A likely: TB10 identified carburetor is Marvel MA-4-5; verify installed carburetor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1" s="48">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>FAA 2012-19-01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Crankshaft replacement</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on engine and crankshaft serial numbers listed in MSB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1" s="48">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>FAA 2015-02-07</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Propeller governor shaft set screws</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>N/A: affects aerobatic wide deck engines; O-360-A1AD is not aerobatic.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1" s="48">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>FAA 2017-16-11</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Connecting rod bushings</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on engine/parts listed in MSB.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1" s="48">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>FAA 2024-21-02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Connecting rod bushings</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>N/A/superseded: control through FAA 2026-04-11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1" s="48">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>FAA 2026-04-11</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Connecting rod bushings</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Uncertain: if affected bushings installed, inspect at every oil change until terminating replacement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1" s="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>FAA 92-12-05</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Piston pin replacement</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on engine S/N or affected piston pin purchase/installation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1" s="48">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>FAA 96-09-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Oil pump impeller replacement</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on sintered iron/aluminium impeller installation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1" s="48">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>FAA 97-15-11</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Piston pin replacement</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Uncertain: depends on engine S/N or cylinder kits installed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1" s="48">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>FAA 98-02-08</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>FAA</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Crankshaft inspection fixed-pitch propellers</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>N/A: TB10 configured with Hartzell constant-speed propeller, not fixed pitch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1" s="48">
+      <c r="A52" s="25" t="n"/>
+      <c r="B52" s="25" t="n"/>
+      <c r="C52" s="25" t="n"/>
+      <c r="D52" s="26" t="n"/>
+      <c r="E52" s="26" t="n"/>
+      <c r="F52" s="26" t="n"/>
+      <c r="G52" s="25" t="n"/>
+      <c r="H52" s="25" t="n"/>
+      <c r="I52" s="25" t="n"/>
+      <c r="J52" s="25" t="n"/>
+      <c r="K52" s="25" t="n"/>
+      <c r="L52" s="25" t="n"/>
+      <c r="M52" s="26" t="n"/>
+    </row>
+    <row r="53" ht="15.75" customHeight="1" s="48">
+      <c r="A53" s="25" t="n"/>
+      <c r="B53" s="25" t="n"/>
+      <c r="C53" s="25" t="n"/>
+      <c r="D53" s="26" t="n"/>
+      <c r="E53" s="26" t="n"/>
+      <c r="F53" s="26" t="n"/>
+      <c r="G53" s="25" t="n"/>
+      <c r="H53" s="25" t="n"/>
+      <c r="I53" s="25" t="n"/>
+      <c r="J53" s="25" t="n"/>
+      <c r="K53" s="25" t="n"/>
+      <c r="L53" s="25" t="n"/>
+      <c r="M53" s="26" t="n"/>
+    </row>
+    <row r="54" ht="15.75" customHeight="1" s="48">
+      <c r="A54" s="25" t="n"/>
+      <c r="B54" s="25" t="n"/>
+      <c r="C54" s="25" t="n"/>
+      <c r="D54" s="26" t="n"/>
+      <c r="E54" s="26" t="n"/>
+      <c r="F54" s="26" t="n"/>
+      <c r="G54" s="25" t="n"/>
+      <c r="H54" s="25" t="n"/>
+      <c r="I54" s="25" t="n"/>
+      <c r="J54" s="25" t="n"/>
+      <c r="K54" s="25" t="n"/>
+      <c r="L54" s="25" t="n"/>
+      <c r="M54" s="26" t="n"/>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="48">
+      <c r="A55" s="25" t="n"/>
+      <c r="B55" s="25" t="n"/>
+      <c r="C55" s="25" t="n"/>
+      <c r="D55" s="26" t="n"/>
+      <c r="E55" s="26" t="n"/>
+      <c r="F55" s="26" t="n"/>
+      <c r="G55" s="25" t="n"/>
+      <c r="H55" s="25" t="n"/>
+      <c r="I55" s="25" t="n"/>
+      <c r="J55" s="25" t="n"/>
+      <c r="K55" s="25" t="n"/>
+      <c r="L55" s="25" t="n"/>
+      <c r="M55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="15.75" customHeight="1" s="48">
+      <c r="A56" s="25" t="n"/>
+      <c r="B56" s="25" t="n"/>
+      <c r="C56" s="25" t="n"/>
+      <c r="D56" s="26" t="n"/>
+      <c r="E56" s="26" t="n"/>
+      <c r="F56" s="26" t="n"/>
+      <c r="G56" s="25" t="n"/>
+      <c r="H56" s="25" t="n"/>
+      <c r="I56" s="25" t="n"/>
+      <c r="J56" s="25" t="n"/>
+      <c r="K56" s="25" t="n"/>
+      <c r="L56" s="25" t="n"/>
+      <c r="M56" s="26" t="n"/>
+    </row>
+    <row r="57" ht="15.75" customHeight="1" s="48">
+      <c r="A57" s="25" t="n"/>
+      <c r="B57" s="25" t="n"/>
+      <c r="C57" s="25" t="n"/>
+      <c r="D57" s="26" t="n"/>
+      <c r="E57" s="26" t="n"/>
+      <c r="F57" s="26" t="n"/>
+      <c r="G57" s="25" t="n"/>
+      <c r="H57" s="25" t="n"/>
+      <c r="I57" s="25" t="n"/>
+      <c r="J57" s="25" t="n"/>
+      <c r="K57" s="25" t="n"/>
+      <c r="L57" s="25" t="n"/>
+      <c r="M57" s="26" t="n"/>
+    </row>
+    <row r="58" ht="15.75" customHeight="1" s="48">
+      <c r="A58" s="25" t="n"/>
+      <c r="B58" s="25" t="n"/>
+      <c r="C58" s="25" t="n"/>
+      <c r="D58" s="25" t="n"/>
+      <c r="E58" s="25" t="n"/>
+      <c r="F58" s="25" t="n"/>
+      <c r="G58" s="25" t="n"/>
+      <c r="H58" s="25" t="n"/>
+      <c r="I58" s="25" t="n"/>
+      <c r="J58" s="25" t="n"/>
+      <c r="K58" s="25" t="n"/>
+      <c r="L58" s="25" t="n"/>
+      <c r="M58" s="26" t="n"/>
+    </row>
+    <row r="59" ht="15.75" customHeight="1" s="48">
+      <c r="A59" s="25" t="n"/>
+      <c r="B59" s="25" t="n"/>
+      <c r="C59" s="25" t="n"/>
+      <c r="D59" s="25" t="n"/>
+      <c r="E59" s="25" t="n"/>
+      <c r="F59" s="25" t="n"/>
+      <c r="G59" s="25" t="n"/>
+      <c r="H59" s="25" t="n"/>
+      <c r="I59" s="25" t="n"/>
+      <c r="J59" s="25" t="n"/>
+      <c r="K59" s="25" t="n"/>
+      <c r="L59" s="25" t="n"/>
+      <c r="M59" s="26" t="n"/>
+    </row>
+    <row r="60" ht="15.75" customHeight="1" s="48">
+      <c r="A60" s="25" t="n"/>
+      <c r="B60" s="25" t="n"/>
+      <c r="C60" s="25" t="n"/>
+      <c r="D60" s="25" t="n"/>
+      <c r="E60" s="25" t="n"/>
+      <c r="F60" s="25" t="n"/>
+      <c r="G60" s="25" t="n"/>
+      <c r="H60" s="25" t="n"/>
+      <c r="I60" s="25" t="n"/>
+      <c r="J60" s="25" t="n"/>
+      <c r="K60" s="25" t="n"/>
+      <c r="L60" s="25" t="n"/>
+      <c r="M60" s="26" t="n"/>
+    </row>
+    <row r="61" ht="15.75" customHeight="1" s="48">
+      <c r="A61" s="25" t="n"/>
+      <c r="B61" s="25" t="n"/>
+      <c r="C61" s="25" t="n"/>
+      <c r="D61" s="25" t="n"/>
+      <c r="E61" s="25" t="n"/>
+      <c r="F61" s="25" t="n"/>
+      <c r="G61" s="25" t="n"/>
+      <c r="H61" s="25" t="n"/>
+      <c r="I61" s="25" t="n"/>
+      <c r="J61" s="25" t="n"/>
+      <c r="K61" s="25" t="n"/>
+      <c r="L61" s="25" t="n"/>
+      <c r="M61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="15.75" customHeight="1" s="48">
+      <c r="A62" s="25" t="n"/>
+      <c r="B62" s="25" t="n"/>
+      <c r="C62" s="25" t="n"/>
+      <c r="D62" s="25" t="n"/>
+      <c r="E62" s="25" t="n"/>
+      <c r="F62" s="25" t="n"/>
+      <c r="G62" s="25" t="n"/>
+      <c r="H62" s="25" t="n"/>
+      <c r="I62" s="25" t="n"/>
+      <c r="J62" s="25" t="n"/>
+      <c r="K62" s="25" t="n"/>
+      <c r="L62" s="25" t="n"/>
+      <c r="M62" s="26" t="n"/>
+    </row>
     <row r="63" ht="15.75" customHeight="1" s="48"/>
     <row r="64" ht="15.75" customHeight="1" s="48"/>
     <row r="65" ht="15.75" customHeight="1" s="48"/>

</xml_diff>

<commit_message>
Finalize rubric review and cleanup
</commit_message>
<xml_diff>
--- a/Control_de_aeronavegabilidad2026.xlsx
+++ b/Control_de_aeronavegabilidad2026.xlsx
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B1" s="67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>EC-SIM</t>
         </is>
       </c>
       <c r="C1" s="67" t="n"/>
@@ -2866,7 +2866,7 @@
     <row r="2">
       <c r="A2" s="71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Airraft Model </t>
+          <t>Aircraft Model</t>
         </is>
       </c>
       <c r="B2" s="71" t="inlineStr">
@@ -2933,7 +2933,7 @@
     <row r="4">
       <c r="A4" s="71" t="inlineStr">
         <is>
-          <t>Manufactura Date (Y)</t>
+          <t>Manufacture Date (Y)</t>
         </is>
       </c>
       <c r="B4" s="71" t="n">
@@ -5588,7 +5588,7 @@
       <c r="B1" s="67" t="n"/>
       <c r="C1" s="67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>EC-SIM</t>
         </is>
       </c>
       <c r="D1" s="67" t="n"/>
@@ -5613,7 +5613,7 @@
     <row r="2">
       <c r="A2" s="71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Airraft Model </t>
+          <t>Aircraft Model</t>
         </is>
       </c>
       <c r="B2" s="72" t="n"/>
@@ -5684,7 +5684,7 @@
     <row r="4">
       <c r="A4" s="71" t="inlineStr">
         <is>
-          <t>Manufactura Date (Y)</t>
+          <t>Manufacture Date (Y)</t>
         </is>
       </c>
       <c r="B4" s="72" t="n"/>
@@ -5813,7 +5813,7 @@
       </c>
       <c r="L7" s="82" t="inlineStr">
         <is>
-          <t>Tipe of Task (OH, Discard, On Condition)</t>
+          <t>Type of Task (OH, Discard, On Condition)</t>
         </is>
       </c>
       <c r="M7" s="82" t="inlineStr">
@@ -6771,7 +6771,7 @@
       </c>
       <c r="L29" s="82" t="inlineStr">
         <is>
-          <t>Tipe of Task (OH, Discard, On Condition)</t>
+          <t>Type of Task (OH, Discard, On Condition)</t>
         </is>
       </c>
       <c r="M29" s="82" t="inlineStr">
@@ -8081,7 +8081,7 @@
       <c r="C1" s="67" t="n"/>
       <c r="D1" s="67" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>EC-SIM</t>
         </is>
       </c>
       <c r="E1" s="67" t="n"/>
@@ -8104,7 +8104,7 @@
     <row r="2">
       <c r="A2" s="71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Model </t>
+          <t>Aircraft Model</t>
         </is>
       </c>
       <c r="B2" s="72" t="n"/>
@@ -8180,7 +8180,7 @@
     <row r="4">
       <c r="A4" s="71" t="inlineStr">
         <is>
-          <t>Manufactura Date (Y)</t>
+          <t>Manufacture Date (Y)</t>
         </is>
       </c>
       <c r="B4" s="72" t="n"/>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="M8" s="86" t="inlineStr">
         <is>
-          <t>Remarcks</t>
+          <t>Remarks</t>
         </is>
       </c>
     </row>
@@ -9062,7 +9062,7 @@
       </c>
       <c r="M28" s="86" t="inlineStr">
         <is>
-          <t>Remarcks</t>
+          <t>Remarks</t>
         </is>
       </c>
     </row>

</xml_diff>